<commit_message>
Deploying to main from @ open-resource-discovery/specification@1429197b121bae6f982e427706ccd0b7adc1d810 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-183/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-183/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="206">
   <si>
     <t>Entity Name</t>
   </si>
@@ -1005,7 +1005,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D480"/>
+  <dimension ref="A1:D478"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -3855,13 +3855,13 @@
         <v>102</v>
       </c>
       <c r="B204" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="C204" t="b">
         <v>0</v>
       </c>
       <c r="D204" t="s">
-        <v>84</v>
+        <v>9</v>
       </c>
     </row>
     <row r="205" spans="1:4" x14ac:dyDescent="0.25">
@@ -3869,7 +3869,7 @@
         <v>102</v>
       </c>
       <c r="B205" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C205" t="b">
         <v>0</v>
@@ -3883,7 +3883,7 @@
         <v>102</v>
       </c>
       <c r="B206" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C206" t="b">
         <v>0</v>
@@ -3897,7 +3897,7 @@
         <v>102</v>
       </c>
       <c r="B207" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C207" t="b">
         <v>0</v>
@@ -3911,13 +3911,13 @@
         <v>102</v>
       </c>
       <c r="B208" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C208" t="b">
         <v>0</v>
       </c>
       <c r="D208" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.25">
@@ -3925,13 +3925,13 @@
         <v>102</v>
       </c>
       <c r="B209" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C209" t="b">
         <v>0</v>
       </c>
       <c r="D209" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.25">
@@ -3939,13 +3939,13 @@
         <v>102</v>
       </c>
       <c r="B210" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="C210" t="b">
         <v>0</v>
       </c>
       <c r="D210" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.25">
@@ -3953,7 +3953,7 @@
         <v>102</v>
       </c>
       <c r="B211" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C211" t="b">
         <v>0</v>
@@ -3967,13 +3967,13 @@
         <v>102</v>
       </c>
       <c r="B212" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C212" t="b">
         <v>0</v>
       </c>
       <c r="D212" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
@@ -3981,32 +3981,32 @@
         <v>102</v>
       </c>
       <c r="B213" t="s">
-        <v>16</v>
+        <v>85</v>
       </c>
       <c r="C213" t="b">
         <v>0</v>
       </c>
       <c r="D213" t="s">
-        <v>9</v>
+        <v>51</v>
       </c>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="B214" t="s">
-        <v>85</v>
+        <v>5</v>
       </c>
       <c r="C214" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D214" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B215" t="s">
         <v>5</v>
@@ -4020,10 +4020,10 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B216" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C216" t="b">
         <v>1</v>
@@ -4037,10 +4037,10 @@
         <v>114</v>
       </c>
       <c r="B217" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C217" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D217" t="s">
         <v>6</v>
@@ -4051,10 +4051,10 @@
         <v>114</v>
       </c>
       <c r="B218" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C218" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D218" t="s">
         <v>6</v>
@@ -4065,7 +4065,7 @@
         <v>114</v>
       </c>
       <c r="B219" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C219" t="b">
         <v>1</v>
@@ -4079,10 +4079,10 @@
         <v>114</v>
       </c>
       <c r="B220" t="s">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="C220" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D220" t="s">
         <v>6</v>
@@ -4093,13 +4093,13 @@
         <v>114</v>
       </c>
       <c r="B221" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C221" t="b">
         <v>0</v>
       </c>
       <c r="D221" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
@@ -4107,24 +4107,24 @@
         <v>114</v>
       </c>
       <c r="B222" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C222" t="b">
         <v>0</v>
       </c>
       <c r="D222" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B223" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="C223" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D223" t="s">
         <v>6</v>
@@ -4135,10 +4135,10 @@
         <v>117</v>
       </c>
       <c r="B224" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C224" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D224" t="s">
         <v>6</v>
@@ -4149,10 +4149,10 @@
         <v>117</v>
       </c>
       <c r="B225" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C225" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D225" t="s">
         <v>6</v>
@@ -4163,7 +4163,7 @@
         <v>117</v>
       </c>
       <c r="B226" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C226" t="b">
         <v>1</v>
@@ -4177,13 +4177,13 @@
         <v>117</v>
       </c>
       <c r="B227" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C227" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D227" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.25">
@@ -4191,13 +4191,13 @@
         <v>117</v>
       </c>
       <c r="B228" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="C228" t="b">
         <v>0</v>
       </c>
       <c r="D228" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.25">
@@ -4205,7 +4205,7 @@
         <v>117</v>
       </c>
       <c r="B229" t="s">
-        <v>38</v>
+        <v>116</v>
       </c>
       <c r="C229" t="b">
         <v>0</v>
@@ -4216,13 +4216,13 @@
     </row>
     <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B230" t="s">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="C230" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D230" t="s">
         <v>6</v>
@@ -4233,10 +4233,10 @@
         <v>118</v>
       </c>
       <c r="B231" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C231" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D231" t="s">
         <v>6</v>
@@ -4247,13 +4247,13 @@
         <v>118</v>
       </c>
       <c r="B232" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C232" t="b">
         <v>0</v>
       </c>
       <c r="D232" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.25">
@@ -4261,13 +4261,13 @@
         <v>118</v>
       </c>
       <c r="B233" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C233" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D233" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="234" spans="1:4" x14ac:dyDescent="0.25">
@@ -4275,10 +4275,10 @@
         <v>118</v>
       </c>
       <c r="B234" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C234" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D234" t="s">
         <v>6</v>
@@ -4289,7 +4289,7 @@
         <v>118</v>
       </c>
       <c r="B235" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C235" t="b">
         <v>0</v>
@@ -4303,7 +4303,7 @@
         <v>118</v>
       </c>
       <c r="B236" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="C236" t="b">
         <v>0</v>
@@ -4317,10 +4317,10 @@
         <v>118</v>
       </c>
       <c r="B237" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C237" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D237" t="s">
         <v>6</v>
@@ -4331,13 +4331,13 @@
         <v>118</v>
       </c>
       <c r="B238" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C238" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D238" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="239" spans="1:4" x14ac:dyDescent="0.25">
@@ -4345,13 +4345,13 @@
         <v>118</v>
       </c>
       <c r="B239" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="C239" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D239" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="240" spans="1:4" x14ac:dyDescent="0.25">
@@ -4359,10 +4359,10 @@
         <v>118</v>
       </c>
       <c r="B240" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C240" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D240" t="s">
         <v>6</v>
@@ -4373,10 +4373,10 @@
         <v>118</v>
       </c>
       <c r="B241" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C241" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D241" t="s">
         <v>6</v>
@@ -4387,7 +4387,7 @@
         <v>118</v>
       </c>
       <c r="B242" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C242" t="b">
         <v>1</v>
@@ -4401,13 +4401,13 @@
         <v>118</v>
       </c>
       <c r="B243" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C243" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D243" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="244" spans="1:4" x14ac:dyDescent="0.25">
@@ -4415,13 +4415,13 @@
         <v>118</v>
       </c>
       <c r="B244" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C244" t="b">
         <v>0</v>
       </c>
       <c r="D244" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="245" spans="1:4" x14ac:dyDescent="0.25">
@@ -4429,13 +4429,13 @@
         <v>118</v>
       </c>
       <c r="B245" t="s">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="C245" t="b">
         <v>0</v>
       </c>
       <c r="D245" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
@@ -4443,13 +4443,13 @@
         <v>118</v>
       </c>
       <c r="B246" t="s">
-        <v>26</v>
+        <v>74</v>
       </c>
       <c r="C246" t="b">
         <v>0</v>
       </c>
       <c r="D246" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
@@ -4457,7 +4457,7 @@
         <v>118</v>
       </c>
       <c r="B247" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C247" t="b">
         <v>0</v>
@@ -4471,7 +4471,7 @@
         <v>118</v>
       </c>
       <c r="B248" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C248" t="b">
         <v>0</v>
@@ -4485,13 +4485,13 @@
         <v>118</v>
       </c>
       <c r="B249" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C249" t="b">
         <v>0</v>
       </c>
       <c r="D249" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
@@ -4499,13 +4499,13 @@
         <v>118</v>
       </c>
       <c r="B250" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C250" t="b">
         <v>0</v>
       </c>
       <c r="D250" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
@@ -4513,13 +4513,13 @@
         <v>118</v>
       </c>
       <c r="B251" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="C251" t="b">
         <v>0</v>
       </c>
       <c r="D251" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.25">
@@ -4527,7 +4527,7 @@
         <v>118</v>
       </c>
       <c r="B252" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C252" t="b">
         <v>0</v>
@@ -4541,7 +4541,7 @@
         <v>118</v>
       </c>
       <c r="B253" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C253" t="b">
         <v>0</v>
@@ -4555,7 +4555,7 @@
         <v>118</v>
       </c>
       <c r="B254" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C254" t="b">
         <v>0</v>
@@ -4569,7 +4569,7 @@
         <v>118</v>
       </c>
       <c r="B255" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="C255" t="b">
         <v>0</v>
@@ -4583,13 +4583,13 @@
         <v>118</v>
       </c>
       <c r="B256" t="s">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="C256" t="b">
         <v>0</v>
       </c>
       <c r="D256" t="s">
-        <v>9</v>
+        <v>120</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
@@ -4597,13 +4597,13 @@
         <v>118</v>
       </c>
       <c r="B257" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C257" t="b">
         <v>0</v>
       </c>
       <c r="D257" t="s">
-        <v>120</v>
+        <v>9</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
@@ -4611,13 +4611,13 @@
         <v>118</v>
       </c>
       <c r="B258" t="s">
-        <v>121</v>
+        <v>19</v>
       </c>
       <c r="C258" t="b">
         <v>0</v>
       </c>
       <c r="D258" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
@@ -4625,13 +4625,13 @@
         <v>118</v>
       </c>
       <c r="B259" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C259" t="b">
         <v>0</v>
       </c>
       <c r="D259" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
@@ -4639,13 +4639,13 @@
         <v>118</v>
       </c>
       <c r="B260" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="C260" t="b">
         <v>0</v>
       </c>
       <c r="D260" t="s">
-        <v>84</v>
+        <v>33</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
@@ -4653,41 +4653,41 @@
         <v>118</v>
       </c>
       <c r="B261" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C261" t="b">
         <v>0</v>
       </c>
       <c r="D261" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B262" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C262" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D262" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B263" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="C263" t="b">
         <v>0</v>
       </c>
       <c r="D263" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
@@ -4695,10 +4695,10 @@
         <v>122</v>
       </c>
       <c r="B264" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C264" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D264" t="s">
         <v>6</v>
@@ -4709,10 +4709,10 @@
         <v>122</v>
       </c>
       <c r="B265" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C265" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D265" t="s">
         <v>6</v>
@@ -4723,7 +4723,7 @@
         <v>122</v>
       </c>
       <c r="B266" t="s">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="C266" t="b">
         <v>0</v>
@@ -4737,7 +4737,7 @@
         <v>122</v>
       </c>
       <c r="B267" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C267" t="b">
         <v>1</v>
@@ -4751,10 +4751,10 @@
         <v>122</v>
       </c>
       <c r="B268" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="C268" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D268" t="s">
         <v>6</v>
@@ -4765,13 +4765,13 @@
         <v>122</v>
       </c>
       <c r="B269" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="C269" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D269" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
@@ -4779,13 +4779,13 @@
         <v>122</v>
       </c>
       <c r="B270" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C270" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D270" t="s">
-        <v>6</v>
+        <v>58</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
@@ -4793,13 +4793,13 @@
         <v>122</v>
       </c>
       <c r="B271" t="s">
-        <v>55</v>
+        <v>94</v>
       </c>
       <c r="C271" t="b">
         <v>0</v>
       </c>
       <c r="D271" t="s">
-        <v>56</v>
+        <v>123</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
@@ -4807,13 +4807,13 @@
         <v>122</v>
       </c>
       <c r="B272" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="C272" t="b">
         <v>0</v>
       </c>
       <c r="D272" t="s">
-        <v>58</v>
+        <v>9</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
@@ -4821,41 +4821,41 @@
         <v>122</v>
       </c>
       <c r="B273" t="s">
-        <v>94</v>
+        <v>32</v>
       </c>
       <c r="C273" t="b">
         <v>0</v>
       </c>
       <c r="D273" t="s">
-        <v>123</v>
+        <v>33</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B274" t="s">
-        <v>31</v>
+        <v>97</v>
       </c>
       <c r="C274" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D274" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B275" t="s">
-        <v>32</v>
+        <v>98</v>
       </c>
       <c r="C275" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D275" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
@@ -4863,7 +4863,7 @@
         <v>124</v>
       </c>
       <c r="B276" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C276" t="b">
         <v>1</v>
@@ -4877,13 +4877,13 @@
         <v>124</v>
       </c>
       <c r="B277" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C277" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D277" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
@@ -4891,10 +4891,10 @@
         <v>124</v>
       </c>
       <c r="B278" t="s">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="C278" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D278" t="s">
         <v>6</v>
@@ -4905,24 +4905,24 @@
         <v>124</v>
       </c>
       <c r="B279" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C279" t="b">
         <v>0</v>
       </c>
       <c r="D279" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B280" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C280" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D280" t="s">
         <v>6</v>
@@ -4930,16 +4930,16 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B281" t="s">
-        <v>116</v>
+        <v>8</v>
       </c>
       <c r="C281" t="b">
         <v>0</v>
       </c>
       <c r="D281" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
@@ -4947,7 +4947,7 @@
         <v>125</v>
       </c>
       <c r="B282" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C282" t="b">
         <v>1</v>
@@ -4961,13 +4961,13 @@
         <v>125</v>
       </c>
       <c r="B283" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C283" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D283" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
@@ -4975,10 +4975,10 @@
         <v>125</v>
       </c>
       <c r="B284" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C284" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D284" t="s">
         <v>6</v>
@@ -4989,7 +4989,7 @@
         <v>125</v>
       </c>
       <c r="B285" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="C285" t="b">
         <v>1</v>
@@ -5003,7 +5003,7 @@
         <v>125</v>
       </c>
       <c r="B286" t="s">
-        <v>12</v>
+        <v>126</v>
       </c>
       <c r="C286" t="b">
         <v>0</v>
@@ -5017,13 +5017,13 @@
         <v>125</v>
       </c>
       <c r="B287" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C287" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D287" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
@@ -5031,13 +5031,13 @@
         <v>125</v>
       </c>
       <c r="B288" t="s">
-        <v>126</v>
+        <v>32</v>
       </c>
       <c r="C288" t="b">
         <v>0</v>
       </c>
       <c r="D288" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
@@ -5045,41 +5045,41 @@
         <v>125</v>
       </c>
       <c r="B289" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C289" t="b">
         <v>0</v>
       </c>
       <c r="D289" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B290" t="s">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="C290" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D290" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B291" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C291" t="b">
         <v>0</v>
       </c>
       <c r="D291" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
@@ -5087,13 +5087,13 @@
         <v>127</v>
       </c>
       <c r="B292" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C292" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D292" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
@@ -5101,10 +5101,10 @@
         <v>127</v>
       </c>
       <c r="B293" t="s">
-        <v>7</v>
+        <v>97</v>
       </c>
       <c r="C293" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D293" t="s">
         <v>6</v>
@@ -5115,13 +5115,13 @@
         <v>127</v>
       </c>
       <c r="B294" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="C294" t="b">
         <v>0</v>
       </c>
       <c r="D294" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
@@ -5129,7 +5129,7 @@
         <v>127</v>
       </c>
       <c r="B295" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="C295" t="b">
         <v>1</v>
@@ -5143,7 +5143,7 @@
         <v>127</v>
       </c>
       <c r="B296" t="s">
-        <v>115</v>
+        <v>11</v>
       </c>
       <c r="C296" t="b">
         <v>0</v>
@@ -5157,10 +5157,10 @@
         <v>127</v>
       </c>
       <c r="B297" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C297" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D297" t="s">
         <v>6</v>
@@ -5171,7 +5171,7 @@
         <v>127</v>
       </c>
       <c r="B298" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="C298" t="b">
         <v>0</v>
@@ -5185,10 +5185,10 @@
         <v>127</v>
       </c>
       <c r="B299" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="C299" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D299" t="s">
         <v>6</v>
@@ -5199,13 +5199,13 @@
         <v>127</v>
       </c>
       <c r="B300" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C300" t="b">
         <v>0</v>
       </c>
       <c r="D300" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
@@ -5213,7 +5213,7 @@
         <v>127</v>
       </c>
       <c r="B301" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C301" t="b">
         <v>1</v>
@@ -5227,13 +5227,13 @@
         <v>127</v>
       </c>
       <c r="B302" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C302" t="b">
         <v>0</v>
       </c>
       <c r="D302" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
@@ -5241,7 +5241,7 @@
         <v>127</v>
       </c>
       <c r="B303" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C303" t="b">
         <v>1</v>
@@ -5255,10 +5255,10 @@
         <v>127</v>
       </c>
       <c r="B304" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="C304" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D304" t="s">
         <v>6</v>
@@ -5269,13 +5269,13 @@
         <v>127</v>
       </c>
       <c r="B305" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="C305" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D305" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
@@ -5283,10 +5283,10 @@
         <v>127</v>
       </c>
       <c r="B306" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C306" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D306" t="s">
         <v>6</v>
@@ -5297,13 +5297,13 @@
         <v>127</v>
       </c>
       <c r="B307" t="s">
-        <v>53</v>
+        <v>92</v>
       </c>
       <c r="C307" t="b">
         <v>0</v>
       </c>
       <c r="D307" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
@@ -5311,13 +5311,13 @@
         <v>127</v>
       </c>
       <c r="B308" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>6</v>
+        <v>56</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
@@ -5325,13 +5325,13 @@
         <v>127</v>
       </c>
       <c r="B309" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
       </c>
       <c r="D309" t="s">
-        <v>9</v>
+        <v>58</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
@@ -5339,13 +5339,13 @@
         <v>127</v>
       </c>
       <c r="B310" t="s">
-        <v>55</v>
+        <v>128</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>56</v>
+        <v>129</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
@@ -5353,13 +5353,13 @@
         <v>127</v>
       </c>
       <c r="B311" t="s">
-        <v>57</v>
+        <v>94</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>58</v>
+        <v>130</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
@@ -5367,13 +5367,13 @@
         <v>127</v>
       </c>
       <c r="B312" t="s">
-        <v>128</v>
+        <v>19</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>129</v>
+        <v>20</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -5381,13 +5381,13 @@
         <v>127</v>
       </c>
       <c r="B313" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>130</v>
+        <v>84</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
@@ -5395,13 +5395,13 @@
         <v>127</v>
       </c>
       <c r="B314" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
@@ -5409,13 +5409,13 @@
         <v>127</v>
       </c>
       <c r="B315" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>84</v>
+        <v>33</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
@@ -5423,13 +5423,13 @@
         <v>127</v>
       </c>
       <c r="B316" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
@@ -5437,41 +5437,41 @@
         <v>127</v>
       </c>
       <c r="B317" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>33</v>
+        <v>51</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B318" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="C318" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D318" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B319" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
@@ -5479,7 +5479,7 @@
         <v>131</v>
       </c>
       <c r="B320" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C320" t="b">
         <v>1</v>
@@ -5493,10 +5493,10 @@
         <v>131</v>
       </c>
       <c r="B321" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C321" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D321" t="s">
         <v>6</v>
@@ -5507,13 +5507,13 @@
         <v>131</v>
       </c>
       <c r="B322" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C322" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D322" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
@@ -5521,10 +5521,10 @@
         <v>131</v>
       </c>
       <c r="B323" t="s">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="C323" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D323" t="s">
         <v>6</v>
@@ -5535,24 +5535,24 @@
         <v>131</v>
       </c>
       <c r="B324" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
       </c>
       <c r="D324" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B325" t="s">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C325" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D325" t="s">
         <v>6</v>
@@ -5560,10 +5560,10 @@
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B326" t="s">
-        <v>116</v>
+        <v>7</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
@@ -5577,13 +5577,13 @@
         <v>132</v>
       </c>
       <c r="B327" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C327" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
@@ -5591,10 +5591,10 @@
         <v>132</v>
       </c>
       <c r="B328" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C328" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D328" t="s">
         <v>6</v>
@@ -5605,13 +5605,13 @@
         <v>132</v>
       </c>
       <c r="B329" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C329" t="b">
         <v>0</v>
       </c>
       <c r="D329" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
@@ -5619,10 +5619,10 @@
         <v>132</v>
       </c>
       <c r="B330" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" t="s">
         <v>6</v>
@@ -5633,10 +5633,10 @@
         <v>132</v>
       </c>
       <c r="B331" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C331" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D331" t="s">
         <v>6</v>
@@ -5647,13 +5647,13 @@
         <v>132</v>
       </c>
       <c r="B332" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C332" t="b">
         <v>0</v>
       </c>
       <c r="D332" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
@@ -5661,7 +5661,7 @@
         <v>132</v>
       </c>
       <c r="B333" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C333" t="b">
         <v>1</v>
@@ -5675,13 +5675,13 @@
         <v>132</v>
       </c>
       <c r="B334" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C334" t="b">
         <v>0</v>
       </c>
       <c r="D334" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
@@ -5689,7 +5689,7 @@
         <v>132</v>
       </c>
       <c r="B335" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C335" t="b">
         <v>1</v>
@@ -5703,10 +5703,10 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="C336" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D336" t="s">
         <v>6</v>
@@ -5717,10 +5717,10 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="C337" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D337" t="s">
         <v>6</v>
@@ -5731,13 +5731,13 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="C338" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D338" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
@@ -5745,13 +5745,13 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>60</v>
+        <v>133</v>
       </c>
       <c r="C339" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D339" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
@@ -5759,13 +5759,13 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>61</v>
+        <v>134</v>
       </c>
       <c r="C340" t="b">
         <v>0</v>
       </c>
       <c r="D340" t="s">
-        <v>9</v>
+        <v>135</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
@@ -5773,13 +5773,13 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C341" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D341" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
@@ -5787,13 +5787,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>134</v>
+        <v>19</v>
       </c>
       <c r="C342" t="b">
         <v>0</v>
       </c>
       <c r="D342" t="s">
-        <v>135</v>
+        <v>20</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5801,7 +5801,7 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>136</v>
+        <v>31</v>
       </c>
       <c r="C343" t="b">
         <v>0</v>
@@ -5815,13 +5815,13 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C344" t="b">
         <v>0</v>
       </c>
       <c r="D344" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
@@ -5829,41 +5829,41 @@
         <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C345" t="b">
         <v>0</v>
       </c>
       <c r="D345" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B346" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B347" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="C347" t="b">
         <v>0</v>
       </c>
       <c r="D347" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
@@ -5871,13 +5871,13 @@
         <v>137</v>
       </c>
       <c r="B348" t="s">
-        <v>10</v>
+        <v>133</v>
       </c>
       <c r="C348" t="b">
         <v>1</v>
       </c>
       <c r="D348" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
@@ -5885,13 +5885,13 @@
         <v>137</v>
       </c>
       <c r="B349" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
       <c r="C349" t="b">
         <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
@@ -5899,13 +5899,13 @@
         <v>137</v>
       </c>
       <c r="B350" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="C350" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>51</v>
+        <v>140</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
@@ -5913,13 +5913,13 @@
         <v>137</v>
       </c>
       <c r="B351" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>51</v>
+        <v>142</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
@@ -5927,13 +5927,13 @@
         <v>137</v>
       </c>
       <c r="B352" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
@@ -5941,41 +5941,41 @@
         <v>137</v>
       </c>
       <c r="B353" t="s">
-        <v>141</v>
+        <v>32</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>142</v>
+        <v>33</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B354" t="s">
-        <v>143</v>
+        <v>5</v>
       </c>
       <c r="C354" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D354" t="s">
-        <v>144</v>
+        <v>6</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B355" t="s">
-        <v>32</v>
+        <v>146</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
@@ -5983,13 +5983,13 @@
         <v>145</v>
       </c>
       <c r="B356" t="s">
-        <v>5</v>
+        <v>147</v>
       </c>
       <c r="C356" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>6</v>
+        <v>148</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
@@ -5997,41 +5997,41 @@
         <v>145</v>
       </c>
       <c r="B357" t="s">
-        <v>146</v>
+        <v>32</v>
       </c>
       <c r="C357" t="b">
         <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B358" t="s">
-        <v>147</v>
+        <v>5</v>
       </c>
       <c r="C358" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D358" t="s">
-        <v>148</v>
+        <v>6</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B359" t="s">
-        <v>32</v>
+        <v>146</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
       </c>
       <c r="D359" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
@@ -6039,13 +6039,13 @@
         <v>149</v>
       </c>
       <c r="B360" t="s">
-        <v>5</v>
+        <v>147</v>
       </c>
       <c r="C360" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>6</v>
+        <v>150</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
@@ -6053,13 +6053,13 @@
         <v>149</v>
       </c>
       <c r="B361" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
@@ -6067,49 +6067,49 @@
         <v>149</v>
       </c>
       <c r="B362" t="s">
-        <v>147</v>
+        <v>32</v>
       </c>
       <c r="C362" t="b">
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>150</v>
+        <v>33</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B363" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C363" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D363" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B364" t="s">
-        <v>32</v>
+        <v>155</v>
       </c>
       <c r="C364" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D364" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B365" t="s">
-        <v>153</v>
+        <v>5</v>
       </c>
       <c r="C365" t="b">
         <v>1</v>
@@ -6120,13 +6120,13 @@
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B366" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="C366" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D366" t="s">
         <v>6</v>
@@ -6137,24 +6137,24 @@
         <v>156</v>
       </c>
       <c r="B367" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C367" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B368" t="s">
-        <v>146</v>
+        <v>5</v>
       </c>
       <c r="C368" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D368" t="s">
         <v>6</v>
@@ -6162,16 +6162,16 @@
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B369" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C369" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D369" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
@@ -6179,13 +6179,13 @@
         <v>157</v>
       </c>
       <c r="B370" t="s">
-        <v>5</v>
+        <v>158</v>
       </c>
       <c r="C370" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
@@ -6193,13 +6193,13 @@
         <v>157</v>
       </c>
       <c r="B371" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C371" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
@@ -6207,13 +6207,13 @@
         <v>157</v>
       </c>
       <c r="B372" t="s">
-        <v>158</v>
+        <v>32</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
@@ -6221,41 +6221,41 @@
         <v>157</v>
       </c>
       <c r="B373" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C373" t="b">
         <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B374" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C374" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D374" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B375" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C375" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D375" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
@@ -6263,7 +6263,7 @@
         <v>159</v>
       </c>
       <c r="B376" t="s">
-        <v>13</v>
+        <v>160</v>
       </c>
       <c r="C376" t="b">
         <v>1</v>
@@ -6277,10 +6277,10 @@
         <v>159</v>
       </c>
       <c r="B377" t="s">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="C377" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D377" t="s">
         <v>6</v>
@@ -6291,10 +6291,10 @@
         <v>159</v>
       </c>
       <c r="B378" t="s">
-        <v>160</v>
+        <v>99</v>
       </c>
       <c r="C378" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D378" t="s">
         <v>6</v>
@@ -6302,13 +6302,13 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B379" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C379" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D379" t="s">
         <v>6</v>
@@ -6316,13 +6316,13 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B380" t="s">
         <v>99</v>
       </c>
       <c r="C380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D380" t="s">
         <v>6</v>
@@ -6333,10 +6333,10 @@
         <v>161</v>
       </c>
       <c r="B381" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C381" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D381" t="s">
         <v>6</v>
@@ -6344,10 +6344,10 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B382" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C382" t="b">
         <v>1</v>
@@ -6358,13 +6358,13 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B383" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D383" t="s">
         <v>6</v>
@@ -6375,10 +6375,10 @@
         <v>162</v>
       </c>
       <c r="B384" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C384" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D384" t="s">
         <v>6</v>
@@ -6389,7 +6389,7 @@
         <v>162</v>
       </c>
       <c r="B385" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C385" t="b">
         <v>1</v>
@@ -6400,13 +6400,13 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B386" t="s">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="C386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D386" t="s">
         <v>6</v>
@@ -6414,13 +6414,13 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B387" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="C387" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D387" t="s">
         <v>6</v>
@@ -6431,7 +6431,7 @@
         <v>163</v>
       </c>
       <c r="B388" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C388" t="b">
         <v>1</v>
@@ -6442,13 +6442,13 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B389" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C389" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D389" t="s">
         <v>6</v>
@@ -6456,13 +6456,13 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B390" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C390" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D390" t="s">
         <v>6</v>
@@ -6473,7 +6473,7 @@
         <v>164</v>
       </c>
       <c r="B391" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C391" t="b">
         <v>1</v>
@@ -6484,13 +6484,13 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B392" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C392" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D392" t="s">
         <v>6</v>
@@ -6498,13 +6498,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B393" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="C393" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6515,7 +6515,7 @@
         <v>165</v>
       </c>
       <c r="B394" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C394" t="b">
         <v>1</v>
@@ -6526,10 +6526,10 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B395" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
       <c r="C395" t="b">
         <v>0</v>
@@ -6540,13 +6540,13 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B396" t="s">
-        <v>99</v>
+        <v>7</v>
       </c>
       <c r="C396" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6557,13 +6557,13 @@
         <v>166</v>
       </c>
       <c r="B397" t="s">
-        <v>167</v>
+        <v>8</v>
       </c>
       <c r="C397" t="b">
         <v>0</v>
       </c>
       <c r="D397" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
@@ -6571,13 +6571,13 @@
         <v>166</v>
       </c>
       <c r="B398" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C398" t="b">
         <v>0</v>
       </c>
       <c r="D398" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
@@ -6585,13 +6585,13 @@
         <v>166</v>
       </c>
       <c r="B399" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C399" t="b">
         <v>0</v>
       </c>
       <c r="D399" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
@@ -6599,35 +6599,35 @@
         <v>166</v>
       </c>
       <c r="B400" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B401" t="s">
-        <v>34</v>
+        <v>169</v>
       </c>
       <c r="C401" t="b">
         <v>0</v>
       </c>
       <c r="D401" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B402" t="s">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="C402" t="b">
         <v>0</v>
@@ -6641,13 +6641,13 @@
         <v>168</v>
       </c>
       <c r="B403" t="s">
-        <v>169</v>
+        <v>32</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
       </c>
       <c r="D403" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
@@ -6655,13 +6655,13 @@
         <v>168</v>
       </c>
       <c r="B404" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C404" t="b">
         <v>0</v>
       </c>
       <c r="D404" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
@@ -6669,41 +6669,41 @@
         <v>168</v>
       </c>
       <c r="B405" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C405" t="b">
         <v>0</v>
       </c>
       <c r="D405" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B406" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
       </c>
       <c r="D406" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B407" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C407" t="b">
         <v>0</v>
       </c>
       <c r="D407" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
@@ -6711,13 +6711,13 @@
         <v>170</v>
       </c>
       <c r="B408" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
@@ -6725,13 +6725,13 @@
         <v>170</v>
       </c>
       <c r="B409" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
@@ -6739,13 +6739,13 @@
         <v>170</v>
       </c>
       <c r="B410" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
@@ -6753,41 +6753,41 @@
         <v>170</v>
       </c>
       <c r="B411" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B412" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="C412" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D412" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B413" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
@@ -6795,10 +6795,10 @@
         <v>171</v>
       </c>
       <c r="B414" t="s">
-        <v>97</v>
+        <v>172</v>
       </c>
       <c r="C414" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D414" t="s">
         <v>6</v>
@@ -6806,13 +6806,13 @@
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B415" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="C415" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D415" t="s">
         <v>6</v>
@@ -6820,10 +6820,10 @@
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B416" t="s">
-        <v>172</v>
+        <v>115</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
@@ -6837,10 +6837,10 @@
         <v>173</v>
       </c>
       <c r="B417" t="s">
-        <v>97</v>
+        <v>172</v>
       </c>
       <c r="C417" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D417" t="s">
         <v>6</v>
@@ -6851,7 +6851,7 @@
         <v>173</v>
       </c>
       <c r="B418" t="s">
-        <v>115</v>
+        <v>174</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
@@ -6862,13 +6862,13 @@
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B419" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C419" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D419" t="s">
         <v>6</v>
@@ -6876,13 +6876,13 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B420" t="s">
-        <v>174</v>
+        <v>10</v>
       </c>
       <c r="C420" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D420" t="s">
         <v>6</v>
@@ -6893,10 +6893,10 @@
         <v>175</v>
       </c>
       <c r="B421" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
       <c r="C421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D421" t="s">
         <v>6</v>
@@ -6907,13 +6907,13 @@
         <v>175</v>
       </c>
       <c r="B422" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
@@ -6921,13 +6921,13 @@
         <v>175</v>
       </c>
       <c r="B423" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
@@ -6935,13 +6935,13 @@
         <v>175</v>
       </c>
       <c r="B424" t="s">
-        <v>32</v>
+        <v>177</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
@@ -6949,38 +6949,38 @@
         <v>175</v>
       </c>
       <c r="B425" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
       </c>
       <c r="D425" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B426" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C426" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D426" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B427" t="s">
-        <v>38</v>
+        <v>176</v>
       </c>
       <c r="C427" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -6991,7 +6991,7 @@
         <v>178</v>
       </c>
       <c r="B428" t="s">
-        <v>179</v>
+        <v>10</v>
       </c>
       <c r="C428" t="b">
         <v>1</v>
@@ -7005,10 +7005,10 @@
         <v>178</v>
       </c>
       <c r="B429" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
       <c r="C429" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D429" t="s">
         <v>6</v>
@@ -7019,13 +7019,13 @@
         <v>178</v>
       </c>
       <c r="B430" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C430" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D430" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
@@ -7033,13 +7033,13 @@
         <v>178</v>
       </c>
       <c r="B431" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C431" t="b">
         <v>0</v>
       </c>
       <c r="D431" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
@@ -7047,13 +7047,13 @@
         <v>178</v>
       </c>
       <c r="B432" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="C432" t="b">
         <v>0</v>
       </c>
       <c r="D432" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
@@ -7061,35 +7061,35 @@
         <v>178</v>
       </c>
       <c r="B433" t="s">
-        <v>8</v>
+        <v>38</v>
       </c>
       <c r="C433" t="b">
         <v>0</v>
       </c>
       <c r="D433" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>178</v>
+        <v>84</v>
       </c>
       <c r="B434" t="s">
-        <v>46</v>
+        <v>180</v>
       </c>
       <c r="C434" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D434" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>178</v>
+        <v>84</v>
       </c>
       <c r="B435" t="s">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
@@ -7100,63 +7100,63 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B436" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C436" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D436" t="s">
-        <v>6</v>
+        <v>183</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="B437" t="s">
-        <v>12</v>
+        <v>184</v>
       </c>
       <c r="C437" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D437" t="s">
-        <v>6</v>
+        <v>185</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B438" t="s">
-        <v>182</v>
+        <v>5</v>
       </c>
       <c r="C438" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D438" t="s">
-        <v>183</v>
+        <v>6</v>
       </c>
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="B439" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C439" t="b">
         <v>1</v>
       </c>
       <c r="D439" t="s">
-        <v>185</v>
+        <v>6</v>
       </c>
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B440" t="s">
         <v>5</v>
@@ -7170,7 +7170,7 @@
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B441" t="s">
         <v>187</v>
@@ -7184,10 +7184,10 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B442" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C442" t="b">
         <v>1</v>
@@ -7198,10 +7198,10 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B443" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C443" t="b">
         <v>1</v>
@@ -7212,7 +7212,7 @@
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B444" t="s">
         <v>97</v>
@@ -7226,10 +7226,10 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B445" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C445" t="b">
         <v>1</v>
@@ -7240,10 +7240,10 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B446" t="s">
-        <v>97</v>
+        <v>5</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7254,10 +7254,10 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B447" t="s">
-        <v>192</v>
+        <v>5</v>
       </c>
       <c r="C447" t="b">
         <v>1</v>
@@ -7268,10 +7268,10 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B448" t="s">
-        <v>5</v>
+        <v>196</v>
       </c>
       <c r="C448" t="b">
         <v>1</v>
@@ -7282,7 +7282,7 @@
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B449" t="s">
         <v>5</v>
@@ -7296,13 +7296,13 @@
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B450" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C450" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D450" t="s">
         <v>6</v>
@@ -7310,7 +7310,7 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B451" t="s">
         <v>5</v>
@@ -7324,7 +7324,7 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B452" t="s">
         <v>198</v>
@@ -7338,7 +7338,7 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B453" t="s">
         <v>5</v>
@@ -7352,7 +7352,7 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B454" t="s">
         <v>198</v>
@@ -7366,7 +7366,7 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B455" t="s">
         <v>5</v>
@@ -7380,7 +7380,7 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B456" t="s">
         <v>198</v>
@@ -7394,7 +7394,7 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B457" t="s">
         <v>5</v>
@@ -7408,10 +7408,10 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B458" t="s">
-        <v>198</v>
+        <v>5</v>
       </c>
       <c r="C458" t="b">
         <v>0</v>
@@ -7422,13 +7422,13 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B459" t="s">
-        <v>5</v>
+        <v>179</v>
       </c>
       <c r="C459" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7439,7 +7439,7 @@
         <v>203</v>
       </c>
       <c r="B460" t="s">
-        <v>5</v>
+        <v>176</v>
       </c>
       <c r="C460" t="b">
         <v>0</v>
@@ -7453,10 +7453,10 @@
         <v>203</v>
       </c>
       <c r="B461" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="C461" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D461" t="s">
         <v>6</v>
@@ -7467,7 +7467,7 @@
         <v>203</v>
       </c>
       <c r="B462" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
       <c r="C462" t="b">
         <v>0</v>
@@ -7478,10 +7478,10 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B463" t="s">
-        <v>204</v>
+        <v>5</v>
       </c>
       <c r="C463" t="b">
         <v>1</v>
@@ -7492,10 +7492,10 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B464" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C464" t="b">
         <v>0</v>
@@ -7509,13 +7509,13 @@
         <v>205</v>
       </c>
       <c r="B465" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C465" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D465" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
@@ -7523,10 +7523,10 @@
         <v>205</v>
       </c>
       <c r="B466" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C466" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D466" t="s">
         <v>6</v>
@@ -7537,13 +7537,13 @@
         <v>205</v>
       </c>
       <c r="B467" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C467" t="b">
         <v>0</v>
       </c>
       <c r="D467" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
@@ -7551,7 +7551,7 @@
         <v>205</v>
       </c>
       <c r="B468" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C468" t="b">
         <v>1</v>
@@ -7565,10 +7565,10 @@
         <v>205</v>
       </c>
       <c r="B469" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C469" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7579,13 +7579,13 @@
         <v>205</v>
       </c>
       <c r="B470" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C470" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D470" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
@@ -7593,7 +7593,7 @@
         <v>205</v>
       </c>
       <c r="B471" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="C471" t="b">
         <v>1</v>
@@ -7607,13 +7607,13 @@
         <v>205</v>
       </c>
       <c r="B472" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
       </c>
       <c r="D472" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
@@ -7621,7 +7621,7 @@
         <v>205</v>
       </c>
       <c r="B473" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C473" t="b">
         <v>1</v>
@@ -7635,10 +7635,10 @@
         <v>205</v>
       </c>
       <c r="B474" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="C474" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7649,13 +7649,13 @@
         <v>205</v>
       </c>
       <c r="B475" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="C475" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D475" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
@@ -7663,13 +7663,13 @@
         <v>205</v>
       </c>
       <c r="B476" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="C476" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D476" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
@@ -7677,13 +7677,13 @@
         <v>205</v>
       </c>
       <c r="B477" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C477" t="b">
         <v>0</v>
       </c>
       <c r="D477" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
@@ -7691,40 +7691,12 @@
         <v>205</v>
       </c>
       <c r="B478" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C478" t="b">
         <v>0</v>
       </c>
       <c r="D478" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A479" t="s">
-        <v>205</v>
-      </c>
-      <c r="B479" t="s">
-        <v>32</v>
-      </c>
-      <c r="C479" t="b">
-        <v>0</v>
-      </c>
-      <c r="D479" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A480" t="s">
-        <v>205</v>
-      </c>
-      <c r="B480" t="s">
-        <v>34</v>
-      </c>
-      <c r="C480" t="b">
-        <v>0</v>
-      </c>
-      <c r="D480" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deploying to main from @ open-resource-discovery/specification@0f1a1013220e833b263c1251700e1143e886b02e 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-183/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-183/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1474" uniqueCount="209">
   <si>
     <t>Entity Name</t>
   </si>
@@ -482,6 +482,15 @@
   </si>
   <si>
     <t>Capability Integration Aspect</t>
+  </si>
+  <si>
+    <t>array&lt;CapabilityIntegrationAspectSubset&gt;</t>
+  </si>
+  <si>
+    <t>Capability Integration Aspect Subset</t>
+  </si>
+  <si>
+    <t>skillName</t>
   </si>
   <si>
     <t>Vendor</t>
@@ -1005,7 +1014,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D478"/>
+  <dimension ref="A1:D491"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5213,13 +5222,13 @@
         <v>127</v>
       </c>
       <c r="B301" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C301" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D301" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
@@ -5227,10 +5236,10 @@
         <v>127</v>
       </c>
       <c r="B302" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C302" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D302" t="s">
         <v>6</v>
@@ -5241,10 +5250,10 @@
         <v>127</v>
       </c>
       <c r="B303" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C303" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D303" t="s">
         <v>6</v>
@@ -5255,7 +5264,7 @@
         <v>127</v>
       </c>
       <c r="B304" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C304" t="b">
         <v>1</v>
@@ -5269,13 +5278,13 @@
         <v>127</v>
       </c>
       <c r="B305" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C305" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D305" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
@@ -5283,13 +5292,13 @@
         <v>127</v>
       </c>
       <c r="B306" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C306" t="b">
         <v>0</v>
       </c>
       <c r="D306" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
@@ -5297,13 +5306,13 @@
         <v>127</v>
       </c>
       <c r="B307" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C307" t="b">
         <v>0</v>
       </c>
       <c r="D307" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
@@ -5311,13 +5320,13 @@
         <v>127</v>
       </c>
       <c r="B308" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
@@ -5325,13 +5334,13 @@
         <v>127</v>
       </c>
       <c r="B309" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
       </c>
       <c r="D309" t="s">
-        <v>58</v>
+        <v>6</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
@@ -5339,13 +5348,13 @@
         <v>127</v>
       </c>
       <c r="B310" t="s">
-        <v>128</v>
+        <v>60</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
       </c>
       <c r="D310" t="s">
-        <v>129</v>
+        <v>6</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
@@ -5353,13 +5362,13 @@
         <v>127</v>
       </c>
       <c r="B311" t="s">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
       </c>
       <c r="D311" t="s">
-        <v>130</v>
+        <v>9</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
@@ -5367,13 +5376,13 @@
         <v>127</v>
       </c>
       <c r="B312" t="s">
-        <v>19</v>
+        <v>62</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -5381,13 +5390,13 @@
         <v>127</v>
       </c>
       <c r="B313" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>84</v>
+        <v>9</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
@@ -5395,13 +5404,13 @@
         <v>127</v>
       </c>
       <c r="B314" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
@@ -5409,13 +5418,13 @@
         <v>127</v>
       </c>
       <c r="B315" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>33</v>
+        <v>58</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
@@ -5423,13 +5432,13 @@
         <v>127</v>
       </c>
       <c r="B316" t="s">
-        <v>34</v>
+        <v>128</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>35</v>
+        <v>129</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
@@ -5437,147 +5446,147 @@
         <v>127</v>
       </c>
       <c r="B317" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B318" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C318" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>6</v>
+        <v>130</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B319" t="s">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B320" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="C320" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>6</v>
+        <v>84</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B321" t="s">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="C321" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D321" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B322" t="s">
-        <v>100</v>
+        <v>28</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
       </c>
       <c r="D322" t="s">
-        <v>101</v>
+        <v>9</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B323" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
       </c>
       <c r="D323" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B324" t="s">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
       </c>
       <c r="D324" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B325" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C325" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D325" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B326" t="s">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B327" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C327" t="b">
         <v>0</v>
@@ -5588,27 +5597,27 @@
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B328" t="s">
-        <v>10</v>
+        <v>85</v>
       </c>
       <c r="C328" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D328" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B329" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="C329" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D329" t="s">
         <v>6</v>
@@ -5616,10 +5625,10 @@
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B330" t="s">
-        <v>12</v>
+        <v>115</v>
       </c>
       <c r="C330" t="b">
         <v>0</v>
@@ -5630,10 +5639,10 @@
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B331" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="C331" t="b">
         <v>1</v>
@@ -5644,38 +5653,38 @@
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B332" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="C332" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D332" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B333" t="s">
-        <v>13</v>
+        <v>100</v>
       </c>
       <c r="C333" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D333" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B334" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C334" t="b">
         <v>0</v>
@@ -5686,13 +5695,13 @@
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B335" t="s">
-        <v>38</v>
+        <v>116</v>
       </c>
       <c r="C335" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D335" t="s">
         <v>6</v>
@@ -5703,7 +5712,7 @@
         <v>132</v>
       </c>
       <c r="B336" t="s">
-        <v>52</v>
+        <v>5</v>
       </c>
       <c r="C336" t="b">
         <v>1</v>
@@ -5717,7 +5726,7 @@
         <v>132</v>
       </c>
       <c r="B337" t="s">
-        <v>60</v>
+        <v>7</v>
       </c>
       <c r="C337" t="b">
         <v>0</v>
@@ -5731,7 +5740,7 @@
         <v>132</v>
       </c>
       <c r="B338" t="s">
-        <v>61</v>
+        <v>8</v>
       </c>
       <c r="C338" t="b">
         <v>0</v>
@@ -5745,13 +5754,13 @@
         <v>132</v>
       </c>
       <c r="B339" t="s">
-        <v>133</v>
+        <v>10</v>
       </c>
       <c r="C339" t="b">
         <v>1</v>
       </c>
       <c r="D339" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
@@ -5759,13 +5768,13 @@
         <v>132</v>
       </c>
       <c r="B340" t="s">
-        <v>134</v>
+        <v>11</v>
       </c>
       <c r="C340" t="b">
         <v>0</v>
       </c>
       <c r="D340" t="s">
-        <v>135</v>
+        <v>6</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
@@ -5773,13 +5782,13 @@
         <v>132</v>
       </c>
       <c r="B341" t="s">
-        <v>136</v>
+        <v>12</v>
       </c>
       <c r="C341" t="b">
         <v>0</v>
       </c>
       <c r="D341" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
@@ -5787,13 +5796,13 @@
         <v>132</v>
       </c>
       <c r="B342" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="C342" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D342" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
@@ -5801,7 +5810,7 @@
         <v>132</v>
       </c>
       <c r="B343" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C343" t="b">
         <v>0</v>
@@ -5815,13 +5824,13 @@
         <v>132</v>
       </c>
       <c r="B344" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="C344" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D344" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
@@ -5829,21 +5838,21 @@
         <v>132</v>
       </c>
       <c r="B345" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C345" t="b">
         <v>0</v>
       </c>
       <c r="D345" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B346" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C346" t="b">
         <v>1</v>
@@ -5854,13 +5863,13 @@
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B347" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="C347" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D347" t="s">
         <v>6</v>
@@ -5868,153 +5877,153 @@
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B348" t="s">
-        <v>133</v>
+        <v>60</v>
       </c>
       <c r="C348" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D348" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B349" t="s">
-        <v>138</v>
+        <v>61</v>
       </c>
       <c r="C349" t="b">
         <v>0</v>
       </c>
       <c r="D349" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B350" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C350" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D350" t="s">
-        <v>140</v>
+        <v>51</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B351" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="C351" t="b">
         <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B352" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C352" t="b">
         <v>0</v>
       </c>
       <c r="D352" t="s">
-        <v>144</v>
+        <v>9</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B353" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="C353" t="b">
         <v>0</v>
       </c>
       <c r="D353" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B354" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C354" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B355" t="s">
-        <v>146</v>
+        <v>32</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B356" t="s">
-        <v>147</v>
+        <v>34</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>148</v>
+        <v>35</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="B357" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C357" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D357" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B358" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C358" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D358" t="s">
         <v>6</v>
@@ -6022,91 +6031,91 @@
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B359" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="C359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D359" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B360" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="C360" t="b">
         <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>150</v>
+        <v>51</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B361" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="C361" t="b">
         <v>0</v>
       </c>
       <c r="D361" t="s">
-        <v>9</v>
+        <v>140</v>
       </c>
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="B362" t="s">
-        <v>32</v>
+        <v>141</v>
       </c>
       <c r="C362" t="b">
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>33</v>
+        <v>142</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="B363" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="C363" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D363" t="s">
-        <v>6</v>
+        <v>144</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="B364" t="s">
-        <v>155</v>
+        <v>32</v>
       </c>
       <c r="C364" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D364" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B365" t="s">
         <v>5</v>
@@ -6120,7 +6129,7 @@
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B366" t="s">
         <v>146</v>
@@ -6134,38 +6143,38 @@
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="B367" t="s">
-        <v>32</v>
+        <v>147</v>
       </c>
       <c r="C367" t="b">
         <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="B368" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C368" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D368" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B369" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C369" t="b">
         <v>1</v>
@@ -6176,66 +6185,66 @@
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B370" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="C370" t="b">
         <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B371" t="s">
-        <v>31</v>
+        <v>147</v>
       </c>
       <c r="C371" t="b">
         <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>9</v>
+        <v>150</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B372" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="C372" t="b">
         <v>0</v>
       </c>
       <c r="D372" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="B373" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C373" t="b">
         <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="B374" t="s">
-        <v>13</v>
+        <v>153</v>
       </c>
       <c r="C374" t="b">
         <v>1</v>
@@ -6246,10 +6255,10 @@
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B375" t="s">
-        <v>52</v>
+        <v>155</v>
       </c>
       <c r="C375" t="b">
         <v>1</v>
@@ -6260,10 +6269,10 @@
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B376" t="s">
-        <v>160</v>
+        <v>5</v>
       </c>
       <c r="C376" t="b">
         <v>1</v>
@@ -6274,10 +6283,10 @@
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B377" t="s">
-        <v>12</v>
+        <v>146</v>
       </c>
       <c r="C377" t="b">
         <v>0</v>
@@ -6288,38 +6297,38 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B378" t="s">
-        <v>99</v>
+        <v>147</v>
       </c>
       <c r="C378" t="b">
         <v>0</v>
       </c>
       <c r="D378" t="s">
-        <v>6</v>
+        <v>157</v>
       </c>
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B379" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C379" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D379" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B380" t="s">
-        <v>99</v>
+        <v>159</v>
       </c>
       <c r="C380" t="b">
         <v>1</v>
@@ -6330,13 +6339,13 @@
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B381" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C381" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D381" t="s">
         <v>6</v>
@@ -6344,7 +6353,7 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B382" t="s">
         <v>10</v>
@@ -6358,69 +6367,69 @@
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B383" t="s">
-        <v>99</v>
+        <v>161</v>
       </c>
       <c r="C383" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D383" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B384" t="s">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C384" t="b">
         <v>0</v>
       </c>
       <c r="D384" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B385" t="s">
-        <v>98</v>
+        <v>32</v>
       </c>
       <c r="C385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D385" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B386" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="C386" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D386" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B387" t="s">
-        <v>115</v>
+        <v>13</v>
       </c>
       <c r="C387" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D387" t="s">
         <v>6</v>
@@ -6428,10 +6437,10 @@
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B388" t="s">
-        <v>99</v>
+        <v>52</v>
       </c>
       <c r="C388" t="b">
         <v>1</v>
@@ -6442,10 +6451,10 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B389" t="s">
-        <v>97</v>
+        <v>163</v>
       </c>
       <c r="C389" t="b">
         <v>1</v>
@@ -6456,10 +6465,10 @@
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B390" t="s">
-        <v>115</v>
+        <v>12</v>
       </c>
       <c r="C390" t="b">
         <v>0</v>
@@ -6470,13 +6479,13 @@
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B391" t="s">
         <v>99</v>
       </c>
       <c r="C391" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D391" t="s">
         <v>6</v>
@@ -6484,10 +6493,10 @@
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B392" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="C392" t="b">
         <v>1</v>
@@ -6498,13 +6507,13 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B393" t="s">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="C393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D393" t="s">
         <v>6</v>
@@ -6512,13 +6521,13 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B394" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C394" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D394" t="s">
         <v>6</v>
@@ -6526,13 +6535,13 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B395" t="s">
-        <v>167</v>
+        <v>10</v>
       </c>
       <c r="C395" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D395" t="s">
         <v>6</v>
@@ -6540,13 +6549,13 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B396" t="s">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="C396" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6554,30 +6563,30 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B397" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C397" t="b">
         <v>0</v>
       </c>
       <c r="D397" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B398" t="s">
-        <v>32</v>
+        <v>98</v>
       </c>
       <c r="C398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D398" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="399" spans="1:4" x14ac:dyDescent="0.25">
@@ -6585,13 +6594,13 @@
         <v>166</v>
       </c>
       <c r="B399" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="C399" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D399" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
@@ -6599,24 +6608,24 @@
         <v>166</v>
       </c>
       <c r="B400" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="C400" t="b">
         <v>0</v>
       </c>
       <c r="D400" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B401" t="s">
-        <v>169</v>
+        <v>99</v>
       </c>
       <c r="C401" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D401" t="s">
         <v>6</v>
@@ -6624,44 +6633,44 @@
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B402" t="s">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="C402" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D402" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="403" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B403" t="s">
-        <v>32</v>
+        <v>115</v>
       </c>
       <c r="C403" t="b">
         <v>0</v>
       </c>
       <c r="D403" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B404" t="s">
-        <v>34</v>
+        <v>99</v>
       </c>
       <c r="C404" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D404" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
@@ -6669,21 +6678,21 @@
         <v>168</v>
       </c>
       <c r="B405" t="s">
-        <v>31</v>
+        <v>97</v>
       </c>
       <c r="C405" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D405" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="406" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B406" t="s">
-        <v>13</v>
+        <v>115</v>
       </c>
       <c r="C406" t="b">
         <v>0</v>
@@ -6694,13 +6703,13 @@
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B407" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C407" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D407" t="s">
         <v>6</v>
@@ -6708,86 +6717,86 @@
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
+        <v>169</v>
+      </c>
+      <c r="B408" t="s">
         <v>170</v>
       </c>
-      <c r="B408" t="s">
-        <v>8</v>
-      </c>
       <c r="C408" t="b">
         <v>0</v>
       </c>
       <c r="D408" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="409" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B409" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C409" t="b">
         <v>0</v>
       </c>
       <c r="D409" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B410" t="s">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="C410" t="b">
         <v>0</v>
       </c>
       <c r="D410" t="s">
-        <v>35</v>
+        <v>9</v>
       </c>
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B411" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C411" t="b">
         <v>0</v>
       </c>
       <c r="D411" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="412" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B412" t="s">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="C412" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D412" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B413" t="s">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
       </c>
       <c r="D413" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
@@ -6806,69 +6815,69 @@
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B415" t="s">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="C415" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B416" t="s">
-        <v>115</v>
+        <v>32</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B417" t="s">
-        <v>172</v>
+        <v>34</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B418" t="s">
-        <v>174</v>
+        <v>31</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B419" t="s">
-        <v>176</v>
+        <v>13</v>
       </c>
       <c r="C419" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D419" t="s">
         <v>6</v>
@@ -6876,13 +6885,13 @@
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B420" t="s">
         <v>10</v>
       </c>
       <c r="C420" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D420" t="s">
         <v>6</v>
@@ -6890,21 +6899,21 @@
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B421" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C421" t="b">
         <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B422" t="s">
         <v>32</v>
@@ -6918,24 +6927,24 @@
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B423" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B424" t="s">
-        <v>177</v>
+        <v>31</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
@@ -6946,13 +6955,13 @@
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B425" t="s">
-        <v>38</v>
+        <v>97</v>
       </c>
       <c r="C425" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D425" t="s">
         <v>6</v>
@@ -6960,13 +6969,13 @@
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B426" t="s">
-        <v>179</v>
+        <v>115</v>
       </c>
       <c r="C426" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D426" t="s">
         <v>6</v>
@@ -6974,13 +6983,13 @@
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B427" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C427" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D427" t="s">
         <v>6</v>
@@ -6988,10 +6997,10 @@
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B428" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="C428" t="b">
         <v>1</v>
@@ -7002,10 +7011,10 @@
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B429" t="s">
-        <v>12</v>
+        <v>115</v>
       </c>
       <c r="C429" t="b">
         <v>0</v>
@@ -7016,30 +7025,30 @@
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B430" t="s">
-        <v>32</v>
+        <v>175</v>
       </c>
       <c r="C430" t="b">
         <v>0</v>
       </c>
       <c r="D430" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B431" t="s">
-        <v>8</v>
+        <v>177</v>
       </c>
       <c r="C431" t="b">
         <v>0</v>
       </c>
       <c r="D431" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
@@ -7047,13 +7056,13 @@
         <v>178</v>
       </c>
       <c r="B432" t="s">
-        <v>46</v>
+        <v>179</v>
       </c>
       <c r="C432" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D432" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
@@ -7061,10 +7070,10 @@
         <v>178</v>
       </c>
       <c r="B433" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="C433" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D433" t="s">
         <v>6</v>
@@ -7072,13 +7081,13 @@
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>84</v>
+        <v>178</v>
       </c>
       <c r="B434" t="s">
-        <v>180</v>
+        <v>12</v>
       </c>
       <c r="C434" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D434" t="s">
         <v>6</v>
@@ -7086,55 +7095,55 @@
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>84</v>
+        <v>178</v>
       </c>
       <c r="B435" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
       </c>
       <c r="D435" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B436" t="s">
-        <v>182</v>
+        <v>8</v>
       </c>
       <c r="C436" t="b">
         <v>0</v>
       </c>
       <c r="D436" t="s">
-        <v>183</v>
+        <v>9</v>
       </c>
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B437" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
-        <v>185</v>
+        <v>9</v>
       </c>
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="B438" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C438" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D438" t="s">
         <v>6</v>
@@ -7142,10 +7151,10 @@
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B439" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="C439" t="b">
         <v>1</v>
@@ -7156,10 +7165,10 @@
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B440" t="s">
-        <v>5</v>
+        <v>179</v>
       </c>
       <c r="C440" t="b">
         <v>1</v>
@@ -7170,10 +7179,10 @@
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B441" t="s">
-        <v>187</v>
+        <v>10</v>
       </c>
       <c r="C441" t="b">
         <v>1</v>
@@ -7184,13 +7193,13 @@
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B442" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="C442" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D442" t="s">
         <v>6</v>
@@ -7198,55 +7207,55 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="B443" t="s">
-        <v>190</v>
+        <v>32</v>
       </c>
       <c r="C443" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D443" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B444" t="s">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="C444" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D444" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B445" t="s">
-        <v>192</v>
+        <v>46</v>
       </c>
       <c r="C445" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D445" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="B446" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C446" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D446" t="s">
         <v>6</v>
@@ -7254,10 +7263,10 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>194</v>
+        <v>84</v>
       </c>
       <c r="B447" t="s">
-        <v>5</v>
+        <v>183</v>
       </c>
       <c r="C447" t="b">
         <v>1</v>
@@ -7268,13 +7277,13 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>195</v>
+        <v>84</v>
       </c>
       <c r="B448" t="s">
-        <v>196</v>
+        <v>12</v>
       </c>
       <c r="C448" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D448" t="s">
         <v>6</v>
@@ -7282,35 +7291,35 @@
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="B449" t="s">
-        <v>5</v>
+        <v>185</v>
       </c>
       <c r="C449" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D449" t="s">
-        <v>6</v>
+        <v>186</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="B450" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="C450" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D450" t="s">
-        <v>6</v>
+        <v>188</v>
       </c>
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="B451" t="s">
         <v>5</v>
@@ -7324,13 +7333,13 @@
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="B452" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C452" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D452" t="s">
         <v>6</v>
@@ -7338,7 +7347,7 @@
     </row>
     <row r="453" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B453" t="s">
         <v>5</v>
@@ -7352,13 +7361,13 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
       <c r="B454" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C454" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D454" t="s">
         <v>6</v>
@@ -7366,10 +7375,10 @@
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B455" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C455" t="b">
         <v>1</v>
@@ -7380,13 +7389,13 @@
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="B456" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C456" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D456" t="s">
         <v>6</v>
@@ -7394,10 +7403,10 @@
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B457" t="s">
-        <v>5</v>
+        <v>97</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7408,13 +7417,13 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B458" t="s">
-        <v>5</v>
+        <v>195</v>
       </c>
       <c r="C458" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D458" t="s">
         <v>6</v>
@@ -7422,13 +7431,13 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B459" t="s">
-        <v>179</v>
+        <v>5</v>
       </c>
       <c r="C459" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D459" t="s">
         <v>6</v>
@@ -7436,13 +7445,13 @@
     </row>
     <row r="460" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B460" t="s">
-        <v>176</v>
+        <v>5</v>
       </c>
       <c r="C460" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D460" t="s">
         <v>6</v>
@@ -7450,10 +7459,10 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B461" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C461" t="b">
         <v>1</v>
@@ -7464,13 +7473,13 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B462" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C462" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D462" t="s">
         <v>6</v>
@@ -7478,13 +7487,13 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B463" t="s">
-        <v>5</v>
+        <v>201</v>
       </c>
       <c r="C463" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D463" t="s">
         <v>6</v>
@@ -7492,13 +7501,13 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B464" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C464" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D464" t="s">
         <v>6</v>
@@ -7506,24 +7515,24 @@
     </row>
     <row r="465" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B465" t="s">
-        <v>8</v>
+        <v>201</v>
       </c>
       <c r="C465" t="b">
         <v>0</v>
       </c>
       <c r="D465" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="466" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B466" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C466" t="b">
         <v>1</v>
@@ -7534,10 +7543,10 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B467" t="s">
-        <v>11</v>
+        <v>201</v>
       </c>
       <c r="C467" t="b">
         <v>0</v>
@@ -7548,10 +7557,10 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B468" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C468" t="b">
         <v>1</v>
@@ -7562,13 +7571,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B469" t="s">
-        <v>45</v>
+        <v>201</v>
       </c>
       <c r="C469" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7579,24 +7588,24 @@
         <v>205</v>
       </c>
       <c r="B470" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="C470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D470" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="471" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B471" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C471" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7604,10 +7613,10 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B472" t="s">
-        <v>37</v>
+        <v>182</v>
       </c>
       <c r="C472" t="b">
         <v>0</v>
@@ -7618,13 +7627,13 @@
     </row>
     <row r="473" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B473" t="s">
-        <v>38</v>
+        <v>179</v>
       </c>
       <c r="C473" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7632,10 +7641,10 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B474" t="s">
-        <v>52</v>
+        <v>207</v>
       </c>
       <c r="C474" t="b">
         <v>1</v>
@@ -7646,57 +7655,239 @@
     </row>
     <row r="475" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B475" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C475" t="b">
         <v>0</v>
       </c>
       <c r="D475" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B476" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C476" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D476" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="477" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B477" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="C477" t="b">
         <v>0</v>
       </c>
       <c r="D477" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="478" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B478" t="s">
+        <v>8</v>
+      </c>
+      <c r="C478" t="b">
+        <v>0</v>
+      </c>
+      <c r="D478" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>208</v>
+      </c>
+      <c r="B479" t="s">
+        <v>10</v>
+      </c>
+      <c r="C479" t="b">
+        <v>1</v>
+      </c>
+      <c r="D479" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>208</v>
+      </c>
+      <c r="B480" t="s">
+        <v>11</v>
+      </c>
+      <c r="C480" t="b">
+        <v>0</v>
+      </c>
+      <c r="D480" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>208</v>
+      </c>
+      <c r="B481" t="s">
+        <v>12</v>
+      </c>
+      <c r="C481" t="b">
+        <v>1</v>
+      </c>
+      <c r="D481" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>208</v>
+      </c>
+      <c r="B482" t="s">
+        <v>45</v>
+      </c>
+      <c r="C482" t="b">
+        <v>1</v>
+      </c>
+      <c r="D482" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>208</v>
+      </c>
+      <c r="B483" t="s">
+        <v>46</v>
+      </c>
+      <c r="C483" t="b">
+        <v>0</v>
+      </c>
+      <c r="D483" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>208</v>
+      </c>
+      <c r="B484" t="s">
+        <v>13</v>
+      </c>
+      <c r="C484" t="b">
+        <v>1</v>
+      </c>
+      <c r="D484" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>208</v>
+      </c>
+      <c r="B485" t="s">
+        <v>37</v>
+      </c>
+      <c r="C485" t="b">
+        <v>0</v>
+      </c>
+      <c r="D485" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>208</v>
+      </c>
+      <c r="B486" t="s">
+        <v>38</v>
+      </c>
+      <c r="C486" t="b">
+        <v>1</v>
+      </c>
+      <c r="D486" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>208</v>
+      </c>
+      <c r="B487" t="s">
+        <v>52</v>
+      </c>
+      <c r="C487" t="b">
+        <v>1</v>
+      </c>
+      <c r="D487" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>208</v>
+      </c>
+      <c r="B488" t="s">
+        <v>19</v>
+      </c>
+      <c r="C488" t="b">
+        <v>0</v>
+      </c>
+      <c r="D488" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>208</v>
+      </c>
+      <c r="B489" t="s">
+        <v>31</v>
+      </c>
+      <c r="C489" t="b">
+        <v>0</v>
+      </c>
+      <c r="D489" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>208</v>
+      </c>
+      <c r="B490" t="s">
+        <v>32</v>
+      </c>
+      <c r="C490" t="b">
+        <v>0</v>
+      </c>
+      <c r="D490" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A491" t="s">
+        <v>208</v>
+      </c>
+      <c r="B491" t="s">
         <v>34</v>
       </c>
-      <c r="C478" t="b">
-        <v>0</v>
-      </c>
-      <c r="D478" t="s">
+      <c r="C491" t="b">
+        <v>0</v>
+      </c>
+      <c r="D491" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>